<commit_message>
feat: add backend database, exporter, and frontend level data for cyberescape game
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,80 +12,123 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="79">
   <si>
     <t>#</t>
   </si>
   <si>
+    <t>Operative ID</t>
+  </si>
+  <si>
     <t>Player</t>
   </si>
   <si>
-    <t>Completed At</t>
+    <t>Status</t>
   </si>
   <si>
     <t>Solved</t>
   </si>
   <si>
-    <t xml:space="preserve">L1.Q1
+    <t xml:space="preserve">Level 1
 Sequence</t>
   </si>
   <si>
-    <t xml:space="preserve">L1.Q2
-Binary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2.Q1
+    <t xml:space="preserve">Level 2
 Caesar</t>
   </si>
   <si>
-    <t xml:space="preserve">L2.Q2
-Atbash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L3.Q1
+    <t xml:space="preserve">Level 3
 LeapSeq</t>
   </si>
   <si>
-    <t xml:space="preserve">L3.Q2
-Vowel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L4.Q1
+    <t xml:space="preserve">Level 4
 Signal</t>
   </si>
   <si>
-    <t xml:space="preserve">L4.Q2
-Hardware</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L5.Q1
+    <t xml:space="preserve">Level 5
 Reverse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L5.Q2
-Base64</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL SOLVING
 TIME</t>
   </si>
   <si>
+    <t>Completed / Updated</t>
+  </si>
+  <si>
+    <t>ddb6d420-a07f-4c27-b884-6e68203b7013</t>
+  </si>
+  <si>
+    <t>aryan kawale</t>
+  </si>
+  <si>
+    <t>COMPLETE</t>
+  </si>
+  <si>
+    <t>10 / 10</t>
+  </si>
+  <si>
+    <t>00:06</t>
+  </si>
+  <si>
+    <t>04:11</t>
+  </si>
+  <si>
+    <t>00:25</t>
+  </si>
+  <si>
+    <t>01:20</t>
+  </si>
+  <si>
+    <t>00:01</t>
+  </si>
+  <si>
+    <t>08:06</t>
+  </si>
+  <si>
+    <t>25/10/2026, 10:02:36 am</t>
+  </si>
+  <si>
+    <t>user-001</t>
+  </si>
+  <si>
     <t>TestPlayer</t>
   </si>
   <si>
+    <t>5 / 5</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>00:47</t>
+  </si>
+  <si>
     <t>24/10/2026, 12:14:57 pm</t>
   </si>
   <si>
-    <t>5 / 5</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>00:47</t>
-  </si>
-  <si>
-    <t>Session #</t>
+    <t>79c6c98e-677b-426e-bbb4-8dccfc7f0564</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
+  </si>
+  <si>
+    <t>25/10/2026, 10:06:07 am</t>
+  </si>
+  <si>
+    <t>c2d058e5-5668-467c-ab3d-bb86b98e785c</t>
+  </si>
+  <si>
+    <t>24/10/2026, 12:24:04 pm</t>
+  </si>
+  <si>
+    <t>Overall Status</t>
   </si>
   <si>
     <t>Q#</t>
@@ -94,7 +137,7 @@
     <t>Challenge</t>
   </si>
   <si>
-    <t>Status</t>
+    <t>Question Status</t>
   </si>
   <si>
     <t>Solving Time</t>
@@ -103,47 +146,122 @@
     <t>Seconds</t>
   </si>
   <si>
-    <t>SESSION-001</t>
+    <t>Timestamp</t>
   </si>
   <si>
     <t>Q1</t>
   </si>
   <si>
+    <t>L1.Q1: Difference Sequence</t>
+  </si>
+  <si>
+    <t>SOLVED</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>L1.Q2: Binary Conversion</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>L2.Q1: Caesar Shift</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>L2.Q2: Atbash Cipher</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>L3.Q1: Variable Leap Sequence</t>
+  </si>
+  <si>
+    <t>Q6</t>
+  </si>
+  <si>
+    <t>L3.Q2: Vowel Progression</t>
+  </si>
+  <si>
+    <t>00:17</t>
+  </si>
+  <si>
+    <t>Q7</t>
+  </si>
+  <si>
+    <t>L4.Q1: Character Frequency Riddle</t>
+  </si>
+  <si>
+    <t>00:08</t>
+  </si>
+  <si>
+    <t>Q8</t>
+  </si>
+  <si>
+    <t>L4.Q2: Hardware Security Riddle</t>
+  </si>
+  <si>
+    <t>01:03</t>
+  </si>
+  <si>
+    <t>Q9</t>
+  </si>
+  <si>
+    <t>L5.Q1: Reverse Clue Decryption</t>
+  </si>
+  <si>
+    <t>00:07</t>
+  </si>
+  <si>
+    <t>Q10</t>
+  </si>
+  <si>
+    <t>L5.Q2: Base64 Escape Keyword</t>
+  </si>
+  <si>
+    <t>00:28</t>
+  </si>
+  <si>
     <t>Sequence Analysis</t>
   </si>
   <si>
-    <t>SOLVED</t>
-  </si>
-  <si>
-    <t>Q2</t>
-  </si>
-  <si>
     <t>Cipher Protocol</t>
   </si>
   <si>
-    <t>Q3</t>
-  </si>
-  <si>
     <t>Letter Sequence</t>
   </si>
   <si>
-    <t>Q4</t>
-  </si>
-  <si>
     <t>Signal Intercept</t>
   </si>
   <si>
-    <t>Q5</t>
-  </si>
-  <si>
     <t>Final Decryption</t>
+  </si>
+  <si>
+    <t>L1: Difference Sequence</t>
+  </si>
+  <si>
+    <t>L2: Caesar Shift</t>
+  </si>
+  <si>
+    <t>L3: Variable Leap Sequence</t>
+  </si>
+  <si>
+    <t>L4: Character Frequency Riddle</t>
+  </si>
+  <si>
+    <t>L5: Reverse Clue Decryption</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -169,14 +287,38 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF22C55E"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF1DE9B6"/>
       <sz val="10"/>
       <name val="Consolas"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF22C55E"/>
-      <sz val="10"/>
+      <sz val="9"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="9"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF8BAABE"/>
+      <sz val="9"/>
       <name val="Consolas"/>
     </font>
   </fonts>
@@ -243,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -266,7 +408,34 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -611,18 +780,20 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,37 +830,28 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>18</v>
@@ -698,22 +860,127 @@
         <v>19</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -727,173 +994,772 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>29</v>
+        <v>47</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>45</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="H3" s="6">
+        <v>251</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>49</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H4" s="2">
+        <v>25</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="6">
+        <v>80</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="6">
+        <v>17</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="2">
+        <v>8</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="6">
+        <v>63</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="2">
+        <v>7</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" s="6">
+        <v>28</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="2">
+        <v>47</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="B22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="2">
-        <v>47</v>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add core game logic, database storage, Excel export, and frontend puzzle UI components
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="87">
   <si>
     <t>#</t>
   </si>
@@ -30,23 +30,23 @@
   </si>
   <si>
     <t xml:space="preserve">Level 1
-Sequence</t>
+Keyboard</t>
   </si>
   <si>
     <t xml:space="preserve">Level 2
-Caesar</t>
+Firewall</t>
   </si>
   <si>
     <t xml:space="preserve">Level 3
-LeapSeq</t>
+Identity</t>
   </si>
   <si>
     <t xml:space="preserve">Level 4
-Signal</t>
+Password</t>
   </si>
   <si>
     <t xml:space="preserve">Level 5
-Reverse</t>
+Locker</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL SOLVING
@@ -107,27 +107,39 @@
     <t>24/10/2026, 12:14:57 pm</t>
   </si>
   <si>
+    <t>6d0f29da-f8d9-4c2b-a756-c1ed7eb2fb44</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>1 / 5</t>
+  </si>
+  <si>
+    <t>00:17</t>
+  </si>
+  <si>
+    <t>25/10/2026, 12:27:12 pm</t>
+  </si>
+  <si>
+    <t>c2d058e5-5668-467c-ab3d-bb86b98e785c</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
+  </si>
+  <si>
+    <t>25/10/2026, 12:20:44 pm</t>
+  </si>
+  <si>
     <t>79c6c98e-677b-426e-bbb4-8dccfc7f0564</t>
   </si>
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>INCOMPLETE</t>
-  </si>
-  <si>
-    <t>0 / 5</t>
-  </si>
-  <si>
-    <t>25/10/2026, 10:06:07 am</t>
-  </si>
-  <si>
-    <t>c2d058e5-5668-467c-ab3d-bb86b98e785c</t>
-  </si>
-  <si>
-    <t>24/10/2026, 12:24:04 pm</t>
-  </si>
-  <si>
     <t>Overall Status</t>
   </si>
   <si>
@@ -188,9 +200,6 @@
     <t>L3.Q2: Vowel Progression</t>
   </si>
   <si>
-    <t>00:17</t>
-  </si>
-  <si>
     <t>Q7</t>
   </si>
   <si>
@@ -255,6 +264,21 @@
   </si>
   <si>
     <t>L5: Reverse Clue Decryption</t>
+  </si>
+  <si>
+    <t>L1: The Encrypted Keyboard</t>
+  </si>
+  <si>
+    <t>L2: The Firewall Escape</t>
+  </si>
+  <si>
+    <t>L3: The Hacker's Identity</t>
+  </si>
+  <si>
+    <t>L4: The Central Server Password</t>
+  </si>
+  <si>
+    <t>L5: The Final Locker Breach</t>
   </si>
 </sst>
 </file>
@@ -429,13 +453,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -780,7 +804,7 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -924,7 +948,7 @@
         <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>26</v>
@@ -939,10 +963,10 @@
         <v>26</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -950,16 +974,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>31</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>26</v>
@@ -980,7 +1004,45 @@
         <v>26</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -994,7 +1056,7 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1016,25 +1078,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1048,13 +1110,13 @@
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>16</v>
@@ -1077,13 +1139,13 @@
         <v>14</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>17</v>
@@ -1106,13 +1168,13 @@
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>45</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
@@ -1135,13 +1197,13 @@
         <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>19</v>
@@ -1164,13 +1226,13 @@
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
@@ -1193,16 +1255,16 @@
         <v>14</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="H7" s="6">
         <v>17</v>
@@ -1222,16 +1284,16 @@
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2">
         <v>8</v>
@@ -1251,16 +1313,16 @@
         <v>14</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H9" s="6">
         <v>63</v>
@@ -1280,16 +1342,16 @@
         <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H10" s="2">
         <v>7</v>
@@ -1309,16 +1371,16 @@
         <v>14</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H11" s="6">
         <v>28</v>
@@ -1338,13 +1400,13 @@
         <v>14</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>26</v>
@@ -1367,13 +1429,13 @@
         <v>14</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>26</v>
@@ -1396,13 +1458,13 @@
         <v>14</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>26</v>
@@ -1425,13 +1487,13 @@
         <v>14</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>26</v>
@@ -1454,13 +1516,13 @@
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>27</v>
@@ -1483,22 +1545,22 @@
         <v>31</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>31</v>
+        <v>77</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>26</v>
+        <v>33</v>
+      </c>
+      <c r="H17" s="6">
+        <v>17</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1508,16 +1570,16 @@
       <c r="B18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F18" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -1527,7 +1589,7 @@
         <v>26</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1541,12 +1603,12 @@
         <v>31</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F19" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="17" t="s">
         <v>31</v>
       </c>
       <c r="G19" s="6" t="s">
@@ -1556,7 +1618,7 @@
         <v>26</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1566,16 +1628,16 @@
       <c r="B20" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F20" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G20" s="2" t="s">
@@ -1585,7 +1647,7 @@
         <v>26</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1599,12 +1661,12 @@
         <v>31</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="17" t="s">
         <v>31</v>
       </c>
       <c r="G21" s="6" t="s">
@@ -1614,26 +1676,26 @@
         <v>26</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F22" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="F22" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G22" s="2" t="s">
@@ -1643,26 +1705,26 @@
         <v>26</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>31</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F23" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F23" s="17" t="s">
         <v>31</v>
       </c>
       <c r="G23" s="6" t="s">
@@ -1672,26 +1734,26 @@
         <v>26</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F24" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G24" s="2" t="s">
@@ -1701,26 +1763,26 @@
         <v>26</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>31</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F25" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="17" t="s">
         <v>31</v>
       </c>
       <c r="G25" s="6" t="s">
@@ -1730,36 +1792,181 @@
         <v>26</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>35</v>
+      <c r="E29" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add frontend authentication, puzzle views, and backend server integration
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -17,10 +17,10 @@
     <t>#</t>
   </si>
   <si>
-    <t>Operative ID</t>
-  </si>
-  <si>
-    <t>Player</t>
+    <t>Team ID</t>
+  </si>
+  <si>
+    <t>Team Name</t>
   </si>
   <si>
     <t>Status</t>

</xml_diff>

<commit_message>
feat: implement core escape room game state hook and utility libraries
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="97">
   <si>
     <t>#</t>
   </si>
@@ -56,15 +56,45 @@
     <t>Completed / Updated</t>
   </si>
   <si>
+    <t>b755f821-0720-48fa-8560-cb80b6b46a66</t>
+  </si>
+  <si>
+    <t>tester</t>
+  </si>
+  <si>
+    <t>COMPLETE</t>
+  </si>
+  <si>
+    <t>5 / 5</t>
+  </si>
+  <si>
+    <t>02:15</t>
+  </si>
+  <si>
+    <t>00:20</t>
+  </si>
+  <si>
+    <t>00:15</t>
+  </si>
+  <si>
+    <t>00:30</t>
+  </si>
+  <si>
+    <t>00:28</t>
+  </si>
+  <si>
+    <t>03:48</t>
+  </si>
+  <si>
+    <t>25/10/2026, 4:40:14 pm</t>
+  </si>
+  <si>
     <t>ddb6d420-a07f-4c27-b884-6e68203b7013</t>
   </si>
   <si>
     <t>aryan kawale</t>
   </si>
   <si>
-    <t>COMPLETE</t>
-  </si>
-  <si>
     <t>10 / 10</t>
   </si>
   <si>
@@ -95,9 +125,6 @@
     <t>TestPlayer</t>
   </si>
   <si>
-    <t>5 / 5</t>
-  </si>
-  <si>
     <t>—</t>
   </si>
   <si>
@@ -107,15 +134,27 @@
     <t>24/10/2026, 12:14:57 pm</t>
   </si>
   <si>
+    <t>a7c49941-ff0c-4534-aeb0-5ee10fa90c13</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
+  </si>
+  <si>
+    <t>25/10/2026, 4:45:49 pm</t>
+  </si>
+  <si>
     <t>6d0f29da-f8d9-4c2b-a756-c1ed7eb2fb44</t>
   </si>
   <si>
     <t>test</t>
   </si>
   <si>
-    <t>INCOMPLETE</t>
-  </si>
-  <si>
     <t>1 / 5</t>
   </si>
   <si>
@@ -128,12 +167,6 @@
     <t>c2d058e5-5668-467c-ab3d-bb86b98e785c</t>
   </si>
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>0 / 5</t>
-  </si>
-  <si>
     <t>25/10/2026, 12:20:44 pm</t>
   </si>
   <si>
@@ -164,33 +197,48 @@
     <t>Q1</t>
   </si>
   <si>
+    <t>L1: The Encrypted Keyboard</t>
+  </si>
+  <si>
+    <t>SOLVED</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>L2: The Firewall Escape</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>L3: The Hacker's Identity</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>L4: The Central Server Password</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>L5: The Final Locker Breach</t>
+  </si>
+  <si>
     <t>L1.Q1: Difference Sequence</t>
   </si>
   <si>
-    <t>SOLVED</t>
-  </si>
-  <si>
-    <t>Q2</t>
-  </si>
-  <si>
     <t>L1.Q2: Binary Conversion</t>
   </si>
   <si>
-    <t>Q3</t>
-  </si>
-  <si>
     <t>L2.Q1: Caesar Shift</t>
   </si>
   <si>
-    <t>Q4</t>
-  </si>
-  <si>
     <t>L2.Q2: Atbash Cipher</t>
   </si>
   <si>
-    <t>Q5</t>
-  </si>
-  <si>
     <t>L3.Q1: Variable Leap Sequence</t>
   </si>
   <si>
@@ -233,9 +281,6 @@
     <t>L5.Q2: Base64 Escape Keyword</t>
   </si>
   <si>
-    <t>00:28</t>
-  </si>
-  <si>
     <t>Sequence Analysis</t>
   </si>
   <si>
@@ -264,21 +309,6 @@
   </si>
   <si>
     <t>L5: Reverse Clue Decryption</t>
-  </si>
-  <si>
-    <t>L1: The Encrypted Keyboard</t>
-  </si>
-  <si>
-    <t>L2: The Firewall Escape</t>
-  </si>
-  <si>
-    <t>L3: The Hacker's Identity</t>
-  </si>
-  <si>
-    <t>L4: The Central Server Password</t>
-  </si>
-  <si>
-    <t>L5: The Final Locker Breach</t>
   </si>
 </sst>
 </file>
@@ -438,10 +468,10 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -450,13 +480,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -804,7 +834,7 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -913,22 +943,22 @@
         <v>26</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -936,37 +966,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -974,37 +1004,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1012,37 +1042,113 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>38</v>
+      <c r="D7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1056,7 +1162,7 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1078,25 +1184,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1110,19 +1216,19 @@
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H2" s="2">
-        <v>6</v>
+        <v>135</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>22</v>
@@ -1139,19 +1245,19 @@
         <v>14</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="H3" s="6">
-        <v>251</v>
+        <v>20</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>22</v>
@@ -1168,19 +1274,19 @@
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>22</v>
@@ -1197,19 +1303,19 @@
         <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>19</v>
       </c>
       <c r="H5" s="6">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>22</v>
@@ -1226,19 +1332,19 @@
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H6" s="2">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>22</v>
@@ -1246,10 +1352,10 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>14</v>
@@ -1258,56 +1364,56 @@
         <v>58</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H7" s="6">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>49</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2">
-        <v>8</v>
+        <v>251</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>14</v>
@@ -1316,77 +1422,77 @@
         <v>63</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="H9" s="6">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="H10" s="2">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>71</v>
+        <v>30</v>
       </c>
       <c r="H11" s="6">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1400,22 +1506,22 @@
         <v>14</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>26</v>
+        <v>46</v>
+      </c>
+      <c r="H12" s="2">
+        <v>17</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1429,22 +1535,22 @@
         <v>14</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>26</v>
+        <v>78</v>
+      </c>
+      <c r="H13" s="6">
+        <v>8</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1458,22 +1564,22 @@
         <v>14</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>26</v>
+        <v>81</v>
+      </c>
+      <c r="H14" s="2">
+        <v>63</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1487,22 +1593,22 @@
         <v>14</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>26</v>
+        <v>84</v>
+      </c>
+      <c r="H15" s="6">
+        <v>7</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1516,457 +1622,747 @@
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H17" s="6">
-        <v>17</v>
+        <v>35</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>31</v>
+        <v>88</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>31</v>
+        <v>89</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>60</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>31</v>
+        <v>90</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>31</v>
+        <v>91</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>60</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>26</v>
+        <v>36</v>
+      </c>
+      <c r="H21" s="6">
+        <v>47</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>31</v>
+        <v>59</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>40</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F24" s="16" t="s">
-        <v>31</v>
+        <v>64</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>40</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>31</v>
+        <v>39</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>31</v>
+        <v>68</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>31</v>
+        <v>44</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>40</v>
       </c>
       <c r="D27" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H27" s="6">
+        <v>17</v>
+      </c>
+      <c r="I27" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>31</v>
+        <v>44</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>31</v>
+        <v>93</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>31</v>
+        <v>44</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>40</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>31</v>
+        <v>44</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F30" s="16" t="s">
-        <v>31</v>
+        <v>95</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>38</v>
+      <c r="C32" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add LeaderboardPage component and vercel routing configuration
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="52">
   <si>
     <t>#</t>
   </si>
@@ -89,81 +89,30 @@
     <t>25/10/2026, 4:40:14 pm</t>
   </si>
   <si>
-    <t>ddb6d420-a07f-4c27-b884-6e68203b7013</t>
-  </si>
-  <si>
-    <t>aryan kawale</t>
-  </si>
-  <si>
-    <t>10 / 10</t>
-  </si>
-  <si>
-    <t>00:06</t>
-  </si>
-  <si>
-    <t>04:11</t>
-  </si>
-  <si>
-    <t>00:25</t>
-  </si>
-  <si>
-    <t>01:20</t>
-  </si>
-  <si>
-    <t>00:01</t>
-  </si>
-  <si>
-    <t>08:06</t>
-  </si>
-  <si>
-    <t>25/10/2026, 10:02:36 am</t>
-  </si>
-  <si>
-    <t>user-001</t>
-  </si>
-  <si>
-    <t>TestPlayer</t>
+    <t>58bb856c-a58a-4a8a-bfe2-63c5382e2134</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
   </si>
   <si>
     <t>—</t>
   </si>
   <si>
-    <t>00:47</t>
-  </si>
-  <si>
-    <t>24/10/2026, 12:14:57 pm</t>
+    <t>25/10/2026, 4:48:02 pm</t>
   </si>
   <si>
     <t>a7c49941-ff0c-4534-aeb0-5ee10fa90c13</t>
   </si>
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>INCOMPLETE</t>
-  </si>
-  <si>
-    <t>0 / 5</t>
-  </si>
-  <si>
     <t>25/10/2026, 4:45:49 pm</t>
   </si>
   <si>
-    <t>6d0f29da-f8d9-4c2b-a756-c1ed7eb2fb44</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>1 / 5</t>
-  </si>
-  <si>
-    <t>00:17</t>
-  </si>
-  <si>
-    <t>25/10/2026, 12:27:12 pm</t>
-  </si>
-  <si>
     <t>c2d058e5-5668-467c-ab3d-bb86b98e785c</t>
   </si>
   <si>
@@ -225,90 +174,6 @@
   </si>
   <si>
     <t>L5: The Final Locker Breach</t>
-  </si>
-  <si>
-    <t>L1.Q1: Difference Sequence</t>
-  </si>
-  <si>
-    <t>L1.Q2: Binary Conversion</t>
-  </si>
-  <si>
-    <t>L2.Q1: Caesar Shift</t>
-  </si>
-  <si>
-    <t>L2.Q2: Atbash Cipher</t>
-  </si>
-  <si>
-    <t>L3.Q1: Variable Leap Sequence</t>
-  </si>
-  <si>
-    <t>Q6</t>
-  </si>
-  <si>
-    <t>L3.Q2: Vowel Progression</t>
-  </si>
-  <si>
-    <t>Q7</t>
-  </si>
-  <si>
-    <t>L4.Q1: Character Frequency Riddle</t>
-  </si>
-  <si>
-    <t>00:08</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>L4.Q2: Hardware Security Riddle</t>
-  </si>
-  <si>
-    <t>01:03</t>
-  </si>
-  <si>
-    <t>Q9</t>
-  </si>
-  <si>
-    <t>L5.Q1: Reverse Clue Decryption</t>
-  </si>
-  <si>
-    <t>00:07</t>
-  </si>
-  <si>
-    <t>Q10</t>
-  </si>
-  <si>
-    <t>L5.Q2: Base64 Escape Keyword</t>
-  </si>
-  <si>
-    <t>Sequence Analysis</t>
-  </si>
-  <si>
-    <t>Cipher Protocol</t>
-  </si>
-  <si>
-    <t>Letter Sequence</t>
-  </si>
-  <si>
-    <t>Signal Intercept</t>
-  </si>
-  <si>
-    <t>Final Decryption</t>
-  </si>
-  <si>
-    <t>L1: Difference Sequence</t>
-  </si>
-  <si>
-    <t>L2: Caesar Shift</t>
-  </si>
-  <si>
-    <t>L3: Variable Leap Sequence</t>
-  </si>
-  <si>
-    <t>L4: Character Frequency Riddle</t>
-  </si>
-  <si>
-    <t>L5: Reverse Clue Decryption</t>
   </si>
 </sst>
 </file>
@@ -439,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -462,13 +327,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -480,16 +342,16 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -834,7 +696,7 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -934,31 +796,31 @@
         <v>24</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>27</v>
       </c>
       <c r="H3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -966,37 +828,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1004,37 +866,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1042,113 +904,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +948,7 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1184,25 +970,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1212,17 +998,17 @@
       <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>60</v>
+        <v>42</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>16</v>
@@ -1241,17 +1027,17 @@
       <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>60</v>
+        <v>45</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>17</v>
@@ -1270,17 +1056,17 @@
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>60</v>
+        <v>47</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
@@ -1299,17 +1085,17 @@
       <c r="B5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>60</v>
+        <v>49</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>19</v>
@@ -1328,17 +1114,17 @@
       <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>60</v>
+        <v>51</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
@@ -1358,25 +1144,25 @@
         <v>24</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>60</v>
+        <v>42</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="6">
-        <v>6</v>
+        <v>27</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1386,26 +1172,26 @@
       <c r="B8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>14</v>
+      <c r="C8" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>60</v>
+        <v>45</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="2">
-        <v>251</v>
+      <c r="H8" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1416,25 +1202,25 @@
         <v>24</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>60</v>
+        <v>47</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="H9" s="6">
-        <v>25</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1444,26 +1230,26 @@
       <c r="B10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>14</v>
+      <c r="C10" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>60</v>
+        <v>49</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" s="2">
-        <v>80</v>
+        <v>27</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1474,895 +1260,460 @@
         <v>24</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>60</v>
+        <v>51</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="6">
-        <v>1</v>
+        <v>27</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>14</v>
+      <c r="C12" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>60</v>
+        <v>42</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12" s="2">
-        <v>17</v>
+        <v>27</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>60</v>
+        <v>45</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H13" s="6">
-        <v>8</v>
+        <v>27</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>14</v>
+      <c r="C14" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>60</v>
+        <v>47</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H14" s="2">
-        <v>63</v>
+        <v>27</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>60</v>
+        <v>49</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="6">
-        <v>7</v>
+        <v>27</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>14</v>
+      <c r="C16" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>60</v>
+        <v>51</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="2">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>60</v>
+        <v>42</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>60</v>
+        <v>45</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>60</v>
+        <v>47</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>60</v>
+        <v>49</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>60</v>
+        <v>51</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="6">
-        <v>47</v>
+        <v>27</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>40</v>
+        <v>45</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F24" s="15" t="s">
-        <v>40</v>
+        <v>47</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>40</v>
+        <v>49</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F26" s="15" t="s">
-        <v>40</v>
+        <v>51</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>25</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="H27" s="6">
-        <v>17</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F28" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I33" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F35" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C37" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F37" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I37" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F38" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F39" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I39" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F40" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F41" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I41" s="6" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add frontend components, styling, levels, and server data for CyberEscape game
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="54">
   <si>
     <t>#</t>
   </si>
@@ -89,19 +89,25 @@
     <t>25/10/2026, 4:40:14 pm</t>
   </si>
   <si>
+    <t>8987ed85-5a53-424e-be48-88597aeceda4</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>25/10/2026, 5:21:47 pm</t>
+  </si>
+  <si>
     <t>58bb856c-a58a-4a8a-bfe2-63c5382e2134</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>INCOMPLETE</t>
-  </si>
-  <si>
-    <t>0 / 5</t>
-  </si>
-  <si>
-    <t>—</t>
   </si>
   <si>
     <t>25/10/2026, 4:48:02 pm</t>
@@ -696,7 +702,7 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -934,7 +940,45 @@
         <v>27</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +992,7 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -970,25 +1014,25 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1002,13 +1046,13 @@
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>16</v>
@@ -1031,13 +1075,13 @@
         <v>14</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>43</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>17</v>
@@ -1060,13 +1104,13 @@
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
@@ -1089,13 +1133,13 @@
         <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>19</v>
@@ -1118,13 +1162,13 @@
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
@@ -1147,10 +1191,10 @@
         <v>25</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>25</v>
@@ -1176,10 +1220,10 @@
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>25</v>
@@ -1205,10 +1249,10 @@
         <v>25</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>25</v>
@@ -1234,10 +1278,10 @@
         <v>25</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F10" s="16" t="s">
         <v>25</v>
@@ -1263,10 +1307,10 @@
         <v>25</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>25</v>
@@ -1292,10 +1336,10 @@
         <v>25</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F12" s="16" t="s">
         <v>25</v>
@@ -1321,10 +1365,10 @@
         <v>25</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>25</v>
@@ -1350,10 +1394,10 @@
         <v>25</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>25</v>
@@ -1379,10 +1423,10 @@
         <v>25</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>25</v>
@@ -1408,10 +1452,10 @@
         <v>25</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>25</v>
@@ -1437,10 +1481,10 @@
         <v>25</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>25</v>
@@ -1466,10 +1510,10 @@
         <v>25</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F18" s="16" t="s">
         <v>25</v>
@@ -1495,10 +1539,10 @@
         <v>25</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>25</v>
@@ -1524,10 +1568,10 @@
         <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>25</v>
@@ -1553,10 +1597,10 @@
         <v>25</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>25</v>
@@ -1582,10 +1626,10 @@
         <v>25</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F22" s="16" t="s">
         <v>25</v>
@@ -1597,7 +1641,7 @@
         <v>27</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1611,10 +1655,10 @@
         <v>25</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F23" s="14" t="s">
         <v>25</v>
@@ -1626,7 +1670,7 @@
         <v>27</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1640,10 +1684,10 @@
         <v>25</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F24" s="16" t="s">
         <v>25</v>
@@ -1655,7 +1699,7 @@
         <v>27</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1669,10 +1713,10 @@
         <v>25</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>25</v>
@@ -1684,7 +1728,7 @@
         <v>27</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1698,22 +1742,167 @@
         <v>25</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>32</v>
+      <c r="F30" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add full-stack React frontend and MongoDB database layer for cyber escape room
</commit_message>
<xml_diff>
--- a/server/cyberEscape_results.xlsx
+++ b/server/cyberEscape_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="72">
   <si>
     <t>#</t>
   </si>
@@ -56,6 +56,132 @@
     <t>Completed / Updated</t>
   </si>
   <si>
+    <t>3551da42-f37c-4fa7-b500-8bacaa9fd23e</t>
+  </si>
+  <si>
+    <t>testerr</t>
+  </si>
+  <si>
+    <t>COMPLETE</t>
+  </si>
+  <si>
+    <t>5 / 5</t>
+  </si>
+  <si>
+    <t>00:09</t>
+  </si>
+  <si>
+    <t>00:12</t>
+  </si>
+  <si>
+    <t>00:17</t>
+  </si>
+  <si>
+    <t>00:14</t>
+  </si>
+  <si>
+    <t>01:04</t>
+  </si>
+  <si>
+    <t>25/10/2026, 8:42:53 pm</t>
+  </si>
+  <si>
+    <t>b209a958-0f05-4100-8b78-ef476e8a1492</t>
+  </si>
+  <si>
+    <t>aryan kawale</t>
+  </si>
+  <si>
+    <t>00:19</t>
+  </si>
+  <si>
+    <t>00:22</t>
+  </si>
+  <si>
+    <t>00:33</t>
+  </si>
+  <si>
+    <t>00:20</t>
+  </si>
+  <si>
+    <t>00:16</t>
+  </si>
+  <si>
+    <t>01:50</t>
+  </si>
+  <si>
+    <t>25/10/2026, 8:06:12 pm</t>
+  </si>
+  <si>
+    <t>8b13b96f-6e33-40a6-9093-8d55f1e97bec</t>
+  </si>
+  <si>
+    <t>test1</t>
+  </si>
+  <si>
+    <t>00:15</t>
+  </si>
+  <si>
+    <t>02:02</t>
+  </si>
+  <si>
+    <t>00:11</t>
+  </si>
+  <si>
+    <t>00:40</t>
+  </si>
+  <si>
+    <t>03:23</t>
+  </si>
+  <si>
+    <t>25/10/2026, 8:31:20 pm</t>
+  </si>
+  <si>
+    <t>3f112539-06f0-4d47-9bae-dd50bc50110a</t>
+  </si>
+  <si>
+    <t>Atifa Sheikh</t>
+  </si>
+  <si>
+    <t>02:45</t>
+  </si>
+  <si>
+    <t>01:42</t>
+  </si>
+  <si>
+    <t>02:25</t>
+  </si>
+  <si>
+    <t>03:57</t>
+  </si>
+  <si>
+    <t>06:30</t>
+  </si>
+  <si>
+    <t>17:19</t>
+  </si>
+  <si>
+    <t>25/10/2026, 8:45:11 pm</t>
+  </si>
+  <si>
+    <t>8fd1baaf-814b-444e-a5ba-1829082e6a62</t>
+  </si>
+  <si>
+    <t>DemoTeam</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>0 / 5</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>25/10/2026, 8:50:41 pm</t>
+  </si>
+  <si>
     <t>Overall Status</t>
   </si>
   <si>
@@ -75,13 +201,46 @@
   </si>
   <si>
     <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>L1: The Encrypted Keyboard</t>
+  </si>
+  <si>
+    <t>SOLVED</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>L2: The Firewall Escape</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>L3: The Hacker's Identity</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>L4: The Central Server Password</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>L5: The Final Locker Breach</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -95,8 +254,54 @@
       <sz val="9"/>
       <name val="Consolas"/>
     </font>
+    <font>
+      <color rgb="FFCDD9E5"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <color rgb="FF1DE9B6"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF22C55E"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1DE9B6"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="10"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF22C55E"/>
+      <sz val="9"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF59E0B"/>
+      <sz val="9"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF8BAABE"/>
+      <sz val="9"/>
+      <name val="Consolas"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -108,8 +313,18 @@
         <fgColor rgb="FF0D1B2A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF071020"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A1628"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -132,14 +347,72 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF16405D"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF16405D"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF16405D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,7 +756,7 @@
   <sheetPr>
     <tabColor rgb="FF35F4D0"/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -534,6 +807,196 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -545,7 +1008,7 @@
   <sheetPr>
     <tabColor rgb="FF1B75BC"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -567,25 +1030,750 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="C2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="6">
+        <v>12</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="2">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="6">
+        <v>17</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="2">
+        <v>14</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="6">
+        <v>19</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2">
+        <v>22</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="6">
+        <v>33</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="2">
+        <v>20</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="6">
+        <v>16</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="2">
         <v>15</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>18</v>
+      <c r="I12" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="6">
+        <v>122</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="2">
+        <v>11</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="6">
+        <v>40</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" s="2">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="6">
+        <v>165</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="2">
+        <v>102</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="6">
+        <v>145</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H20" s="2">
+        <v>237</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H21" s="6">
+        <v>390</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>